<commit_message>
added tests + methods
</commit_message>
<xml_diff>
--- a/Errorlogs.xlsx
+++ b/Errorlogs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preci\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FA56425-7F83-41B6-A435-C73F62761A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DB9C869-762A-4BE5-84C0-4281BD08455F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3FF41096-B411-4518-97A4-EF687E09AF74}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="64">
   <si>
     <t>Error Log</t>
   </si>
@@ -390,6 +390,26 @@
   </si>
   <si>
     <t>dummyArray.pop()</t>
+  </si>
+  <si>
+    <t>import DummyPy
+def test_answer():
+    assert DummyPy.checkValid() == 8</t>
+  </si>
+  <si>
+    <t>def test_answer():
+&gt;       assert DummyPy.checkValid() == 8
+               ^^^^^^^^^^^^^^^^^^
+E       AttributeError: module 'DummyPy' has no attribute 'checkValid'</t>
+  </si>
+  <si>
+    <t>import DummyPy
+class TestCases:
+    def test_answer(self):
+        assert DummyPy.Solution.checkVaild(self) == 8</t>
+  </si>
+  <si>
+    <t>self means an instance of so it must be in a class to work</t>
   </si>
 </sst>
 </file>
@@ -458,8 +478,7 @@
   </cellStyles>
   <dxfs count="7">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="bottom" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -471,7 +490,8 @@
       <alignment vertical="bottom" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="bottom" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -493,18 +513,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4BED1189-F361-4ACA-BEA3-DC19E8D17ADF}" name="Table1" displayName="Table1" ref="A1:F21" totalsRowShown="0" dataDxfId="6">
-  <autoFilter ref="A1:F21" xr:uid="{4BED1189-F361-4ACA-BEA3-DC19E8D17ADF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4BED1189-F361-4ACA-BEA3-DC19E8D17ADF}" name="Table1" displayName="Table1" ref="A1:F38" totalsRowShown="0" dataDxfId="6">
+  <autoFilter ref="A1:F38" xr:uid="{4BED1189-F361-4ACA-BEA3-DC19E8D17ADF}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F10">
     <sortCondition ref="A1:A10"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{5F2D2825-205B-4C2F-B511-B503548F46F2}" name="Date(dd/mm/yyyy)" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{E2CEFFAE-2F3D-4469-8E32-A32A2DF6A0D3}" name="Resource" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{E04E0E9F-ECB9-46F3-809D-0F065D7412C9}" name="Error Log" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{16101023-7EC6-46D9-9989-AFE42DEF889A}" name="Relevant Code" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{68E20E21-0163-4D3E-9CF1-5EBCD84DCFAE}" name="Solution" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{311E8290-7723-44CE-BF86-7383DE912B10}" name="Reason" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{E2CEFFAE-2F3D-4469-8E32-A32A2DF6A0D3}" name="Resource" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{E04E0E9F-ECB9-46F3-809D-0F065D7412C9}" name="Error Log" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{16101023-7EC6-46D9-9989-AFE42DEF889A}" name="Relevant Code" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{68E20E21-0163-4D3E-9CF1-5EBCD84DCFAE}" name="Solution" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{311E8290-7723-44CE-BF86-7383DE912B10}" name="Reason" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -827,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B0F5737-2136-44EA-B950-84115FEAE98E}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
@@ -1122,7 +1142,9 @@
       <c r="A16" s="3">
         <v>46178</v>
       </c>
-      <c r="B16" s="3"/>
+      <c r="B16" s="3" t="s">
+        <v>45</v>
+      </c>
       <c r="C16" s="1" t="s">
         <v>57</v>
       </c>
@@ -1134,19 +1156,29 @@
       </c>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="116" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
-        <v>46178</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+        <v>46179</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="1"/>
@@ -1156,7 +1188,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="1"/>
@@ -1166,7 +1198,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="1"/>
@@ -1176,13 +1208,165 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B22" s="3"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B26" s="3"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="1"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="1"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="1"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="1"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="1"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="1"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="1"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="1"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="1"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
arrays + lists + string methods
</commit_message>
<xml_diff>
--- a/Errorlogs.xlsx
+++ b/Errorlogs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preci\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DB9C869-762A-4BE5-84C0-4281BD08455F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F098282-57E3-4A59-AF19-93087E391A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3FF41096-B411-4518-97A4-EF687E09AF74}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="74">
   <si>
     <t>Error Log</t>
   </si>
@@ -410,6 +410,46 @@
   </si>
   <si>
     <t>self means an instance of so it must be in a class to work</t>
+  </si>
+  <si>
+    <t>C:\Users\preci\Practice\HelpFuncConsoleApp\HelpFunctions\Program.cs(102,24): error CS1929: 'string' does not contain a
+definition for 'Append' and the best extension method overload 'Queryable.Append&lt;string&gt;(IQueryable&lt;string&gt;, string)' r
+equires a receiver of type 'System.Linq.IQueryable&lt;string&gt;' [C:\Users\preci\Practice\HelpFuncConsoleApp\HelpFunctions\H
+elpFunctions.csproj]</t>
+  </si>
+  <si>
+    <t>String house = "chair is comfy with an execptional mattress";
+            String i = house.Append("fgewf");</t>
+  </si>
+  <si>
+    <t>String house = "chair is comfy with an execptional mattress";
+            String i = "On a very comfy ";
+            i = house + "fgewf";</t>
+  </si>
+  <si>
+    <t>Append doesn't work with strings</t>
+  </si>
+  <si>
+    <t>dummyArray = [1,2,3,4,5,6,7,8,9]
+j = list(dummyArray)
+print(j.count)</t>
+  </si>
+  <si>
+    <t>&lt;built-in method count of list object at 0x000002787AD09D00&gt;</t>
+  </si>
+  <si>
+    <t>print(j.count(100))</t>
+  </si>
+  <si>
+    <t>It takes in value and serches its number of occurences</t>
+  </si>
+  <si>
+    <t>s = "HC"
+        s.lower()</t>
+  </si>
+  <si>
+    <t>s = "HC"
+        s = s.lower()</t>
   </si>
 </sst>
 </file>
@@ -1176,39 +1216,61 @@
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="174" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
-        <v>46179</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46180</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B19" s="3"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C19" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
+      <c r="D20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="F20" s="1"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="1"/>
@@ -1218,7 +1280,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="1"/>
@@ -1228,7 +1290,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="1"/>
@@ -1238,7 +1300,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="1"/>
@@ -1248,7 +1310,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="1"/>
@@ -1258,7 +1320,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="1"/>
@@ -1268,7 +1330,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="1"/>
@@ -1278,7 +1340,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="1"/>
@@ -1288,7 +1350,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="1"/>

</xml_diff>

<commit_message>
classes + constructors + fields
</commit_message>
<xml_diff>
--- a/Errorlogs.xlsx
+++ b/Errorlogs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preci\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F098282-57E3-4A59-AF19-93087E391A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67983E32-4D6C-4F6C-8AFC-664996CD233B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3FF41096-B411-4518-97A4-EF687E09AF74}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="85">
   <si>
     <t>Error Log</t>
   </si>
@@ -450,6 +450,83 @@
   <si>
     <t>s = "HC"
         s = s.lower()</t>
+  </si>
+  <si>
+    <t>C:\Users\preci\Practice\ReturnProject\app\src\main\java\returnproject&gt;javac DummyJava.java
+DummyJava.java:95: error: cannot find symbol
+        System.out.println(new App().count());  symbol:   class App
+  location: class DummyJava
+1 error</t>
+  </si>
+  <si>
+    <t>Enter name:
+Exception in thread "main" java.util.NoSuchElementException: No line found
+        at java.base/java.util.Scanner.nextLine(Scanner.java:1660)
+        at returnproject.DummyJava.main(DummyJava.java:102)</t>
+  </si>
+  <si>
+    <t>public static void main(String [] args){
+        Scanner myScanner = new Scanner(System.in);
+        System.out.println("Enter name: ");
+        String name = myScanner.nextLine();
+        System.out.println(name);
+    }</t>
+  </si>
+  <si>
+    <t>Was running DummyJava.java in isolation so App.java wasn't getting run. Instead, run .\gradlew run as it ensures all files run and in the correct order.</t>
+  </si>
+  <si>
+    <t>build.gradle.kts: application {
+    // Define the main class for the application.
+    mainClass = "returnproject.App"
+} DummyJava.java: package returnproject;
+import java.util.ArrayList;
+public class DummyJava{
+    public static boolean doCalc(){public static void main(String [] args){   System.out.println(new App().count());
+        //System.out.println(j);
+    }}}</t>
+  </si>
+  <si>
+    <t>application {
+    // Define the main class for the application.
+    mainClass = "returnproject.DummyJava"
+} then run .\gradlew run</t>
+  </si>
+  <si>
+    <t>In build.gradle.kts ad: 
+tasks.named&lt;JavaExec&gt;("run") {
+    standardInput = System.`in`
+}</t>
+  </si>
+  <si>
+    <t>Gradle doesn't automatically connect the standard input so there is no input stream for your Scanner.nextLine(). you have to do it manually add it to gradle.</t>
+  </si>
+  <si>
+    <t>File "C:\Users\preci\Practice\ReturnForms\DummyPy2.py", line 6, in Solution2
+    john = Solution2("John", 160)
+           ^^^^^^^^^
+NameError: name 'Solution2' is not defined</t>
+  </si>
+  <si>
+    <t>class Solution2:
+    def __init__(self, age, height):
+        self.age = age
+        self.height = height
+    john = Solution2("John", 160)
+    def getBread(self):
+        return "erfgf"
+mySolution2 = Solution2()
+print(mySolution2.getBread())</t>
+  </si>
+  <si>
+    <t>class Solution2:
+    def __init__(self, age, height):
+        self.age = age
+        self.height = height
+    def getBread(self):
+        return "erfgf" 
+mySolution2 = Solution2("john", 160)
+print(mySolution2.getBread())</t>
   </si>
 </sst>
 </file>
@@ -893,7 +970,7 @@
     <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.6328125" customWidth="1"/>
+    <col min="4" max="4" width="32.453125" customWidth="1"/>
     <col min="5" max="5" width="24.08984375" customWidth="1"/>
     <col min="6" max="6" width="38.90625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1240,7 +1317,9 @@
       <c r="A19" s="3">
         <v>46180</v>
       </c>
-      <c r="B19" s="3"/>
+      <c r="B19" s="3" t="s">
+        <v>45</v>
+      </c>
       <c r="C19" s="1" t="s">
         <v>69</v>
       </c>
@@ -1258,7 +1337,9 @@
       <c r="A20" s="3">
         <v>46180</v>
       </c>
-      <c r="B20" s="3"/>
+      <c r="B20" s="3" t="s">
+        <v>45</v>
+      </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1" t="s">
         <v>72</v>
@@ -1268,39 +1349,67 @@
       </c>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
-        <v>46180</v>
-      </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46181</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
-        <v>46180</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46181</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
-        <v>46180</v>
-      </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
+        <v>46181</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="F23" s="1"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="1"/>
@@ -1310,7 +1419,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="1"/>
@@ -1320,7 +1429,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="1"/>
@@ -1330,7 +1439,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="1"/>
@@ -1340,7 +1449,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="1"/>
@@ -1350,7 +1459,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="1"/>

</xml_diff>

<commit_message>
rewrite progress from memory
</commit_message>
<xml_diff>
--- a/Errorlogs.xlsx
+++ b/Errorlogs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preci\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67983E32-4D6C-4F6C-8AFC-664996CD233B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E1BDBB-0E51-48E2-B159-91998EB06A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3FF41096-B411-4518-97A4-EF687E09AF74}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="102">
   <si>
     <t>Error Log</t>
   </si>
@@ -527,6 +527,173 @@
         return "erfgf" 
 mySolution2 = Solution2("john", 160)
 print(mySolution2.getBread())</t>
+  </si>
+  <si>
+    <t>required: String,int
+    found:    no arguments
+    reason: actual and formal argument lists differ in length
+  C:\Users\preci\Practice2\JavaProject\app\src\main\java\javaproject\App.java:24: error: incompatible types: int cannot be converted to String
+              return testInt;</t>
+  </si>
+  <si>
+    <t>public String getGreeting() {
+        int testInt = 15;
+        if (testInt &gt; 15){
+            testInt *= 4;
+            return testInt;</t>
+  </si>
+  <si>
+    <t>C:\Users\preci\Practice2\CSharpProject&gt;dotnet run
+C:\Users\preci\Practice2\CSharpProject\Program.cs(2,13): error CS1002: ; expected [C:\Users\preci\Practice2\CSharpProje
+ct\CSharpProject.csproj]
+The build failed. Fix the build errors and run again.</t>
+  </si>
+  <si>
+    <t>using System
+namespace CSharpProject
+{
+    internal class Program{
+        static void main(String [] args){
+            Console.WriteLine("Hello World");
+        }
+    }
+}</t>
+  </si>
+  <si>
+    <t>CSC : error CS5001: Program does not contain a static 'Main' method suitable for an entry point [C:\Users\preci\Practic
+e2\CSharpProject\CSharpProject.csproj]</t>
+  </si>
+  <si>
+    <t>static void main(String [] args){
+            Console.WriteLine(ysl * police);
+        }</t>
+  </si>
+  <si>
+    <t>Main' not 'main'</t>
+  </si>
+  <si>
+    <r>
+      <t>using System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">static void </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ain(String [] args){
+            Console.WriteLine(ysl * police);
+        }</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">public String getGreeting() {
+        int testInt = 15;
+        if (testInt &gt; 15){
+            testInt *= 4;
+            return </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>String.valueOf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(testInt);</t>
+    </r>
+  </si>
+  <si>
+    <t>C:\Users\preci\Practice2\CSharpProject\Program.cs(8,9): error CS0825: The contextual keyword 'var' may only appear with
+in a local variable declaration or in script code [C:\Users\preci\Practice2\CSharpProject\CSharpProject.csproj]
+The build failed. Fix the build errors and run again.</t>
+  </si>
+  <si>
+    <t>using System;
+namespace CSharpProject
+{
+    internal class Program{
+        var car = "cars3"</t>
+  </si>
+  <si>
+    <t>public String getCode(){
+            var jupiter = "fgb";
+            return " ";
+        }</t>
+  </si>
+  <si>
+    <t>Can't exist on its own must be in a scope/method</t>
+  </si>
+  <si>
+    <t>C:\Users\preci\Practice2\CSharpProject\Program.cs(52,35): error CS0119: 'string' is a type, which is not valid in the g
+iven context [C:\Users\preci\Practice2\CSharpProject\CSharpProject.csproj]</t>
+  </si>
+  <si>
+    <t>String [] testArray = String[3];</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">String [] testArray = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>new</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> String[3];</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -630,8 +797,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4BED1189-F361-4ACA-BEA3-DC19E8D17ADF}" name="Table1" displayName="Table1" ref="A1:F38" totalsRowShown="0" dataDxfId="6">
-  <autoFilter ref="A1:F38" xr:uid="{4BED1189-F361-4ACA-BEA3-DC19E8D17ADF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4BED1189-F361-4ACA-BEA3-DC19E8D17ADF}" name="Table1" displayName="Table1" ref="A1:F39" totalsRowShown="0" dataDxfId="6">
+  <autoFilter ref="A1:F39" xr:uid="{4BED1189-F361-4ACA-BEA3-DC19E8D17ADF}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F10">
     <sortCondition ref="A1:A10"/>
   </sortState>
@@ -964,11 +1131,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B0F5737-2136-44EA-B950-84115FEAE98E}">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.26953125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.453125" customWidth="1"/>
     <col min="5" max="5" width="24.08984375" customWidth="1"/>
@@ -1407,59 +1574,103 @@
       </c>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
-        <v>46181</v>
-      </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
+        <v>46182</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
-        <v>46181</v>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46182</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
-        <v>46181</v>
-      </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
+        <v>46182</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" ht="116" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
-        <v>46181</v>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46182</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
-        <v>46181</v>
-      </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
+        <v>46182</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>101</v>
+      </c>
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="1"/>
@@ -1468,7 +1679,9 @@
       <c r="F29" s="1"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="1"/>
+      <c r="A30" s="3">
+        <v>46182</v>
+      </c>
       <c r="B30" s="3"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -1476,7 +1689,9 @@
       <c r="F30" s="1"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="1"/>
+      <c r="A31" s="3">
+        <v>46182</v>
+      </c>
       <c r="B31" s="3"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -1484,7 +1699,9 @@
       <c r="F31" s="1"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="1"/>
+      <c r="A32" s="3">
+        <v>46182</v>
+      </c>
       <c r="B32" s="3"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -1492,7 +1709,9 @@
       <c r="F32" s="1"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="1"/>
+      <c r="A33" s="3">
+        <v>46182</v>
+      </c>
       <c r="B33" s="3"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -1500,7 +1719,9 @@
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" s="1"/>
+      <c r="A34" s="3">
+        <v>46182</v>
+      </c>
       <c r="B34" s="3"/>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -1508,7 +1729,9 @@
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" s="1"/>
+      <c r="A35" s="3">
+        <v>46182</v>
+      </c>
       <c r="B35" s="3"/>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -1516,7 +1739,9 @@
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" s="1"/>
+      <c r="A36" s="3">
+        <v>46182</v>
+      </c>
       <c r="B36" s="3"/>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -1524,7 +1749,9 @@
       <c r="F36" s="1"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" s="1"/>
+      <c r="A37" s="3">
+        <v>46182</v>
+      </c>
       <c r="B37" s="3"/>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -1532,12 +1759,24 @@
       <c r="F37" s="1"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" s="1"/>
+      <c r="A38" s="3">
+        <v>46182</v>
+      </c>
       <c r="B38" s="3"/>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="3">
+        <v>46182</v>
+      </c>
+      <c r="B39" s="3"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
rebuilt all prjects + encapsulation + accessmodifiers
</commit_message>
<xml_diff>
--- a/Errorlogs.xlsx
+++ b/Errorlogs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preci\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E1BDBB-0E51-48E2-B159-91998EB06A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A03A41D-835C-4CB0-BBF0-840F34BE84C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3FF41096-B411-4518-97A4-EF687E09AF74}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="106">
   <si>
     <t>Error Log</t>
   </si>
@@ -694,6 +694,49 @@
       </rPr>
       <t xml:space="preserve"> String[3];</t>
     </r>
+  </si>
+  <si>
+    <t>interface InnerDummyJava {
+    public String getSound();
+}                                                                                   public String getSound(String machine){
+        if (machine.toLowerCase().contains("car 
+        ...
+        return " ";
+    }</t>
+  </si>
+  <si>
+    <t>C:\Users\preci\Practice\ReturnProject\app\src\main\java\returnproject\DummyJava.java:15: error: DummyJava is not abstract and does not override abstract method getSound() in InnerDummyJava
+public class DummyJava implements InnerDummyJava, InnerDummyJava_2{</t>
+  </si>
+  <si>
+    <r>
+      <t>interface InnerDummyJava {
+    public String getSound(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>String machine</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>);
+}</t>
+    </r>
+  </si>
+  <si>
+    <t>Basically must be theame with the method defined in the interface</t>
   </si>
 </sst>
 </file>
@@ -1668,19 +1711,29 @@
       </c>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
-        <v>46182</v>
-      </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
+        <v>46184</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="1"/>
@@ -1690,7 +1743,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="1"/>
@@ -1700,7 +1753,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="1"/>
@@ -1710,7 +1763,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="1"/>
@@ -1720,7 +1773,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="1"/>
@@ -1730,7 +1783,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="1"/>
@@ -1740,7 +1793,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="1"/>
@@ -1750,7 +1803,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="1"/>
@@ -1760,7 +1813,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="1"/>
@@ -1770,7 +1823,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="1"/>

</xml_diff>

<commit_message>
exceptions + custom exceptions
</commit_message>
<xml_diff>
--- a/Errorlogs.xlsx
+++ b/Errorlogs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preci\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A03A41D-835C-4CB0-BBF0-840F34BE84C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{703E0983-6D4F-4577-883E-823C1743F223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3FF41096-B411-4518-97A4-EF687E09AF74}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="110">
   <si>
     <t>Error Log</t>
   </si>
@@ -737,6 +737,42 @@
   </si>
   <si>
     <t>Basically must be theame with the method defined in the interface</t>
+  </si>
+  <si>
+    <t>Unhandled exception type Exception</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if (num &lt; 10) {
+            throw new Exception("You're not old enough for this ride.");
+        } </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">throw new </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ArithmeticException</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>("You're not old enough for this ride.");</t>
+    </r>
+  </si>
+  <si>
+    <t>Exception types matter</t>
   </si>
 </sst>
 </file>
@@ -1731,19 +1767,29 @@
         <v>105</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
-        <v>46184</v>
-      </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
+        <v>46185</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="1"/>
@@ -1753,7 +1799,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="1"/>
@@ -1763,7 +1809,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="1"/>
@@ -1773,7 +1819,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="1"/>
@@ -1783,7 +1829,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="1"/>
@@ -1793,7 +1839,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="1"/>
@@ -1803,7 +1849,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="1"/>
@@ -1813,7 +1859,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="1"/>
@@ -1823,7 +1869,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="1"/>

</xml_diff>